<commit_message>
update perubahanan penamaan sheet
</commit_message>
<xml_diff>
--- a/data/UAT Scenarios - PRJ20260044 - BSI BYOND.xlsx
+++ b/data/UAT Scenarios - PRJ20260044 - BSI BYOND.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_MUF - ADITYO\04 Projects\01 Projects\2026\149 PRJ20260044 - BSI BYOND\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_QA_UAT_Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F351791-03D2-47F9-9635-7D2F0BB21858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B5D61D-C840-466E-9989-0B1F5E4DC6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="MAPPING MD &amp; SKENARIO" sheetId="12" r:id="rId1"/>
     <sheet name="MATRIX KONTRAK" sheetId="10" r:id="rId2"/>
     <sheet name="TEST CASES" sheetId="13" r:id="rId3"/>
-    <sheet name="DASHBOARD PROGRESS" sheetId="3" r:id="rId4"/>
+    <sheet name="Dashboard Progress" sheetId="3" r:id="rId4"/>
     <sheet name="DEFECT LOG" sheetId="8" r:id="rId5"/>
     <sheet name="PANDUAN" sheetId="9" r:id="rId6"/>
     <sheet name="LOOKUP" sheetId="4" r:id="rId7"/>
@@ -5115,22 +5115,19 @@
     <xf numFmtId="2" fontId="14" fillId="13" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -5151,29 +5148,35 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -5183,9 +5186,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7636,123 +7636,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40">
-      <c r="A1" s="145" t="s">
+      <c r="A1" s="144" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="145"/>
-      <c r="C1" s="145"/>
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
     </row>
     <row r="2" spans="1:40" ht="16.2" thickBot="1">
-      <c r="A2" s="146"/>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
+      <c r="A2" s="145"/>
+      <c r="B2" s="145"/>
+      <c r="C2" s="145"/>
     </row>
     <row r="3" spans="1:40">
-      <c r="A3" s="151" t="s">
+      <c r="A3" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="153" t="s">
+      <c r="B3" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="153" t="s">
+      <c r="C3" s="139" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="153" t="s">
+      <c r="D3" s="139" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="156" t="s">
+      <c r="E3" s="141" t="s">
         <v>1035</v>
       </c>
-      <c r="F3" s="153" t="s">
+      <c r="F3" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="G3" s="153" t="s">
+      <c r="G3" s="139" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="153" t="s">
+      <c r="H3" s="139" t="s">
         <v>75</v>
       </c>
-      <c r="I3" s="153" t="s">
+      <c r="I3" s="139" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="153" t="s">
+      <c r="J3" s="139" t="s">
         <v>77</v>
       </c>
-      <c r="K3" s="153" t="s">
+      <c r="K3" s="139" t="s">
         <v>78</v>
       </c>
-      <c r="L3" s="153" t="s">
+      <c r="L3" s="139" t="s">
         <v>79</v>
       </c>
-      <c r="M3" s="153" t="s">
+      <c r="M3" s="139" t="s">
         <v>80</v>
       </c>
-      <c r="N3" s="153" t="s">
+      <c r="N3" s="139" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="153" t="s">
+      <c r="O3" s="139" t="s">
         <v>34</v>
       </c>
-      <c r="P3" s="153" t="s">
+      <c r="P3" s="139" t="s">
         <v>82</v>
       </c>
-      <c r="Q3" s="153"/>
-      <c r="R3" s="153"/>
-      <c r="S3" s="153" t="s">
+      <c r="Q3" s="139"/>
+      <c r="R3" s="139"/>
+      <c r="S3" s="139" t="s">
         <v>83</v>
       </c>
-      <c r="T3" s="153"/>
-      <c r="U3" s="153"/>
-      <c r="V3" s="153" t="s">
+      <c r="T3" s="139"/>
+      <c r="U3" s="139"/>
+      <c r="V3" s="139" t="s">
         <v>84</v>
       </c>
-      <c r="W3" s="153" t="s">
+      <c r="W3" s="139" t="s">
         <v>85</v>
       </c>
-      <c r="X3" s="153"/>
-      <c r="Y3" s="153"/>
-      <c r="Z3" s="153" t="s">
+      <c r="X3" s="139"/>
+      <c r="Y3" s="139"/>
+      <c r="Z3" s="139" t="s">
         <v>86</v>
       </c>
-      <c r="AA3" s="153" t="s">
+      <c r="AA3" s="139" t="s">
         <v>87</v>
       </c>
-      <c r="AB3" s="153"/>
-      <c r="AC3" s="153" t="s">
+      <c r="AB3" s="139"/>
+      <c r="AC3" s="139" t="s">
         <v>88</v>
       </c>
-      <c r="AD3" s="153"/>
-      <c r="AE3" s="153"/>
-      <c r="AF3" s="153"/>
-      <c r="AG3" s="153"/>
-      <c r="AH3" s="153"/>
-      <c r="AI3" s="153"/>
-      <c r="AJ3" s="153" t="s">
+      <c r="AD3" s="139"/>
+      <c r="AE3" s="139"/>
+      <c r="AF3" s="139"/>
+      <c r="AG3" s="139"/>
+      <c r="AH3" s="139"/>
+      <c r="AI3" s="139"/>
+      <c r="AJ3" s="139" t="s">
         <v>89</v>
       </c>
-      <c r="AK3" s="153"/>
-      <c r="AL3" s="153"/>
-      <c r="AM3" s="153" t="s">
+      <c r="AK3" s="139"/>
+      <c r="AL3" s="139"/>
+      <c r="AM3" s="139" t="s">
         <v>90</v>
       </c>
-      <c r="AN3" s="155"/>
+      <c r="AN3" s="143"/>
     </row>
     <row r="4" spans="1:40" ht="31.2">
-      <c r="A4" s="152"/>
-      <c r="B4" s="154"/>
-      <c r="C4" s="154"/>
-      <c r="D4" s="154"/>
-      <c r="E4" s="157"/>
-      <c r="F4" s="154"/>
-      <c r="G4" s="154"/>
-      <c r="H4" s="154"/>
-      <c r="I4" s="154"/>
-      <c r="J4" s="154"/>
-      <c r="K4" s="154"/>
-      <c r="L4" s="154"/>
-      <c r="M4" s="154"/>
-      <c r="N4" s="154"/>
-      <c r="O4" s="154"/>
+      <c r="A4" s="153"/>
+      <c r="B4" s="140"/>
+      <c r="C4" s="140"/>
+      <c r="D4" s="140"/>
+      <c r="E4" s="142"/>
+      <c r="F4" s="140"/>
+      <c r="G4" s="140"/>
+      <c r="H4" s="140"/>
+      <c r="I4" s="140"/>
+      <c r="J4" s="140"/>
+      <c r="K4" s="140"/>
+      <c r="L4" s="140"/>
+      <c r="M4" s="140"/>
+      <c r="N4" s="140"/>
+      <c r="O4" s="140"/>
       <c r="P4" s="82" t="s">
         <v>91</v>
       </c>
@@ -7771,7 +7771,7 @@
       <c r="U4" s="82" t="s">
         <v>96</v>
       </c>
-      <c r="V4" s="154"/>
+      <c r="V4" s="140"/>
       <c r="W4" s="82" t="s">
         <v>97</v>
       </c>
@@ -7781,7 +7781,7 @@
       <c r="Y4" s="82" t="s">
         <v>98</v>
       </c>
-      <c r="Z4" s="154"/>
+      <c r="Z4" s="140"/>
       <c r="AA4" s="82" t="s">
         <v>99</v>
       </c>
@@ -10436,131 +10436,131 @@
       </c>
     </row>
     <row r="45" spans="1:40" ht="34.200000000000003" customHeight="1">
-      <c r="A45" s="147" t="s">
+      <c r="A45" s="146" t="s">
         <v>199</v>
       </c>
-      <c r="B45" s="147"/>
-      <c r="C45" s="147"/>
-      <c r="D45" s="141" t="s">
+      <c r="B45" s="146"/>
+      <c r="C45" s="146"/>
+      <c r="D45" s="157" t="s">
         <v>200</v>
       </c>
-      <c r="E45" s="141"/>
-      <c r="F45" s="141"/>
-      <c r="G45" s="141"/>
+      <c r="E45" s="157"/>
+      <c r="F45" s="157"/>
+      <c r="G45" s="157"/>
     </row>
     <row r="46" spans="1:40" ht="16.2" thickBot="1">
-      <c r="A46" s="148"/>
-      <c r="B46" s="148"/>
-      <c r="C46" s="148"/>
+      <c r="A46" s="147"/>
+      <c r="B46" s="147"/>
+      <c r="C46" s="147"/>
     </row>
     <row r="47" spans="1:40">
-      <c r="A47" s="149" t="s">
+      <c r="A47" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="139" t="s">
+      <c r="B47" s="150" t="s">
         <v>70</v>
       </c>
-      <c r="C47" s="139" t="s">
+      <c r="C47" s="150" t="s">
         <v>71</v>
       </c>
-      <c r="D47" s="139" t="s">
+      <c r="D47" s="150" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="143"/>
-      <c r="F47" s="139" t="s">
+      <c r="E47" s="154"/>
+      <c r="F47" s="150" t="s">
         <v>73</v>
       </c>
-      <c r="G47" s="139" t="s">
+      <c r="G47" s="150" t="s">
         <v>201</v>
       </c>
-      <c r="H47" s="139" t="s">
+      <c r="H47" s="150" t="s">
         <v>202</v>
       </c>
-      <c r="I47" s="139" t="s">
+      <c r="I47" s="150" t="s">
         <v>74</v>
       </c>
-      <c r="J47" s="139" t="s">
+      <c r="J47" s="150" t="s">
         <v>75</v>
       </c>
-      <c r="K47" s="139" t="s">
+      <c r="K47" s="150" t="s">
         <v>76</v>
       </c>
-      <c r="L47" s="139" t="s">
+      <c r="L47" s="150" t="s">
         <v>77</v>
       </c>
-      <c r="M47" s="139" t="s">
+      <c r="M47" s="150" t="s">
         <v>78</v>
       </c>
-      <c r="N47" s="139" t="s">
+      <c r="N47" s="150" t="s">
         <v>79</v>
       </c>
-      <c r="O47" s="139" t="s">
+      <c r="O47" s="150" t="s">
         <v>80</v>
       </c>
-      <c r="P47" s="139" t="s">
+      <c r="P47" s="150" t="s">
         <v>81</v>
       </c>
-      <c r="Q47" s="139" t="s">
+      <c r="Q47" s="150" t="s">
         <v>34</v>
       </c>
-      <c r="R47" s="139" t="s">
+      <c r="R47" s="150" t="s">
         <v>82</v>
       </c>
-      <c r="S47" s="139"/>
-      <c r="T47" s="139"/>
-      <c r="U47" s="139" t="s">
+      <c r="S47" s="150"/>
+      <c r="T47" s="150"/>
+      <c r="U47" s="150" t="s">
         <v>83</v>
       </c>
-      <c r="V47" s="139"/>
-      <c r="W47" s="139"/>
-      <c r="X47" s="139" t="s">
+      <c r="V47" s="150"/>
+      <c r="W47" s="150"/>
+      <c r="X47" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="Y47" s="139" t="s">
+      <c r="Y47" s="150" t="s">
         <v>85</v>
       </c>
-      <c r="Z47" s="139"/>
-      <c r="AA47" s="139"/>
-      <c r="AB47" s="139" t="s">
+      <c r="Z47" s="150"/>
+      <c r="AA47" s="150"/>
+      <c r="AB47" s="150" t="s">
         <v>86</v>
       </c>
-      <c r="AC47" s="139" t="s">
+      <c r="AC47" s="150" t="s">
         <v>87</v>
       </c>
-      <c r="AD47" s="139"/>
-      <c r="AE47" s="139" t="s">
+      <c r="AD47" s="150"/>
+      <c r="AE47" s="150" t="s">
         <v>88</v>
       </c>
-      <c r="AF47" s="139"/>
-      <c r="AG47" s="139"/>
-      <c r="AH47" s="139"/>
-      <c r="AI47" s="139"/>
-      <c r="AJ47" s="139"/>
-      <c r="AK47" s="139"/>
-      <c r="AL47" s="139" t="s">
+      <c r="AF47" s="150"/>
+      <c r="AG47" s="150"/>
+      <c r="AH47" s="150"/>
+      <c r="AI47" s="150"/>
+      <c r="AJ47" s="150"/>
+      <c r="AK47" s="150"/>
+      <c r="AL47" s="150" t="s">
         <v>89</v>
       </c>
-      <c r="AM47" s="139"/>
-      <c r="AN47" s="140"/>
+      <c r="AM47" s="150"/>
+      <c r="AN47" s="156"/>
     </row>
     <row r="48" spans="1:40" ht="28.8">
-      <c r="A48" s="150"/>
-      <c r="B48" s="142"/>
-      <c r="C48" s="142"/>
-      <c r="D48" s="142"/>
-      <c r="E48" s="144"/>
-      <c r="F48" s="142"/>
-      <c r="G48" s="142"/>
-      <c r="H48" s="142"/>
-      <c r="I48" s="142"/>
-      <c r="J48" s="142"/>
-      <c r="K48" s="142"/>
-      <c r="L48" s="142"/>
-      <c r="M48" s="142"/>
-      <c r="N48" s="142"/>
-      <c r="O48" s="142"/>
-      <c r="P48" s="142"/>
-      <c r="Q48" s="142"/>
+      <c r="A48" s="149"/>
+      <c r="B48" s="151"/>
+      <c r="C48" s="151"/>
+      <c r="D48" s="151"/>
+      <c r="E48" s="155"/>
+      <c r="F48" s="151"/>
+      <c r="G48" s="151"/>
+      <c r="H48" s="151"/>
+      <c r="I48" s="151"/>
+      <c r="J48" s="151"/>
+      <c r="K48" s="151"/>
+      <c r="L48" s="151"/>
+      <c r="M48" s="151"/>
+      <c r="N48" s="151"/>
+      <c r="O48" s="151"/>
+      <c r="P48" s="151"/>
+      <c r="Q48" s="151"/>
       <c r="R48" s="106" t="s">
         <v>91</v>
       </c>
@@ -10579,7 +10579,7 @@
       <c r="W48" s="106" t="s">
         <v>96</v>
       </c>
-      <c r="X48" s="142"/>
+      <c r="X48" s="151"/>
       <c r="Y48" s="106" t="s">
         <v>97</v>
       </c>
@@ -10589,7 +10589,7 @@
       <c r="AA48" s="106" t="s">
         <v>98</v>
       </c>
-      <c r="AB48" s="142"/>
+      <c r="AB48" s="151"/>
       <c r="AC48" s="106" t="s">
         <v>99</v>
       </c>
@@ -16435,42 +16435,6 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="AM3:AN3"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="Z3:Z4"/>
-    <mergeCell ref="AJ3:AL3"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="S3:U3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="AC3:AI3"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="A45:C46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="N47:N48"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="H47:H48"/>
-    <mergeCell ref="I47:I48"/>
-    <mergeCell ref="E47:E48"/>
     <mergeCell ref="AL47:AN47"/>
     <mergeCell ref="D45:G45"/>
     <mergeCell ref="X47:X48"/>
@@ -16487,6 +16451,42 @@
     <mergeCell ref="K47:K48"/>
     <mergeCell ref="L47:L48"/>
     <mergeCell ref="M47:M48"/>
+    <mergeCell ref="N47:N48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="A45:C46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="AM3:AN3"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="Z3:Z4"/>
+    <mergeCell ref="AJ3:AL3"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="S3:U3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="AC3:AI3"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16524,10 +16524,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="162" t="s">
+      <c r="A1" s="159" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="162"/>
+      <c r="B1" s="159"/>
       <c r="C1" s="104"/>
       <c r="D1" s="70"/>
       <c r="E1" s="70"/>
@@ -16545,11 +16545,11 @@
       <c r="Q1" s="71"/>
     </row>
     <row r="2" spans="1:18" ht="15" customHeight="1" thickBot="1">
-      <c r="A2" s="162" t="s">
+      <c r="A2" s="159" t="s">
         <v>260</v>
       </c>
-      <c r="B2" s="162"/>
-      <c r="C2" s="162"/>
+      <c r="B2" s="159"/>
+      <c r="C2" s="159"/>
       <c r="D2" s="70"/>
       <c r="E2" s="70"/>
       <c r="F2" s="70"/>
@@ -30910,7 +30910,7 @@
       <c r="B316" s="120" t="s">
         <v>1058</v>
       </c>
-      <c r="C316" s="159" t="s">
+      <c r="C316" s="160" t="s">
         <v>152</v>
       </c>
       <c r="D316" s="92" t="s">
@@ -30957,7 +30957,7 @@
       <c r="B317" s="120" t="s">
         <v>1059</v>
       </c>
-      <c r="C317" s="160"/>
+      <c r="C317" s="161"/>
       <c r="D317" s="92" t="s">
         <v>6</v>
       </c>
@@ -31002,7 +31002,7 @@
       <c r="B318" s="120" t="s">
         <v>1060</v>
       </c>
-      <c r="C318" s="161"/>
+      <c r="C318" s="162"/>
       <c r="D318" s="92" t="s">
         <v>8</v>
       </c>
@@ -31100,28 +31100,12 @@
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="C131:C142"/>
-    <mergeCell ref="C45:C56"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C4:C15"/>
-    <mergeCell ref="C16:C32"/>
-    <mergeCell ref="C33:C44"/>
-    <mergeCell ref="C57:C68"/>
-    <mergeCell ref="C69:C87"/>
-    <mergeCell ref="C88:C99"/>
-    <mergeCell ref="C100:C111"/>
-    <mergeCell ref="C112:C130"/>
-    <mergeCell ref="C240:C242"/>
-    <mergeCell ref="C243:C245"/>
-    <mergeCell ref="C246:C248"/>
-    <mergeCell ref="C249:C251"/>
-    <mergeCell ref="C143:C154"/>
-    <mergeCell ref="C234:C236"/>
-    <mergeCell ref="C155:C167"/>
-    <mergeCell ref="C168:C178"/>
-    <mergeCell ref="C179:C194"/>
-    <mergeCell ref="C237:C239"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C312:C313"/>
+    <mergeCell ref="C314:C315"/>
+    <mergeCell ref="C316:C318"/>
+    <mergeCell ref="C300:C303"/>
+    <mergeCell ref="C304:C307"/>
+    <mergeCell ref="C308:C311"/>
     <mergeCell ref="C296:C299"/>
     <mergeCell ref="C252:C254"/>
     <mergeCell ref="C255:C256"/>
@@ -31134,15 +31118,31 @@
     <mergeCell ref="C278:C283"/>
     <mergeCell ref="C284:C286"/>
     <mergeCell ref="C287:C290"/>
+    <mergeCell ref="C240:C242"/>
+    <mergeCell ref="C243:C245"/>
+    <mergeCell ref="C246:C248"/>
+    <mergeCell ref="C249:C251"/>
+    <mergeCell ref="C143:C154"/>
+    <mergeCell ref="C234:C236"/>
+    <mergeCell ref="C155:C167"/>
+    <mergeCell ref="C168:C178"/>
+    <mergeCell ref="C179:C194"/>
+    <mergeCell ref="C237:C239"/>
     <mergeCell ref="C195:C205"/>
     <mergeCell ref="C206:C216"/>
     <mergeCell ref="C217:C233"/>
-    <mergeCell ref="C312:C313"/>
-    <mergeCell ref="C314:C315"/>
-    <mergeCell ref="C316:C318"/>
-    <mergeCell ref="C300:C303"/>
-    <mergeCell ref="C304:C307"/>
-    <mergeCell ref="C308:C311"/>
+    <mergeCell ref="C131:C142"/>
+    <mergeCell ref="C45:C56"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C4:C15"/>
+    <mergeCell ref="C16:C32"/>
+    <mergeCell ref="C33:C44"/>
+    <mergeCell ref="C57:C68"/>
+    <mergeCell ref="C69:C87"/>
+    <mergeCell ref="C88:C99"/>
+    <mergeCell ref="C100:C111"/>
+    <mergeCell ref="C112:C130"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31168,7 +31168,7 @@
     <col min="9" max="16384" width="8.88671875" style="66"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8">
+    <row r="1" spans="1:7">
       <c r="A1" s="67" t="s">
         <v>0</v>
       </c>

</xml_diff>